<commit_message>
DO 8.3 / SO 4.3: RoRo-terrein tegen de kade, fasegrenzen ingekort, dieptelijnen buiten de haven
- RoRo-terrein, -13,70-ligplaatsvak, opstelzone, PDI-hal en laadstraat 200 m terug naar
  het westen: oostrand = RoRo-kade, schip ligt in het -13,70-vak, terrein niet meer in het water
- Fasegrenzen F1|F2 en F2|F3 eindigen op de containerkade (stonden 420 m in de insteek)
- Maatlijn RoRo-kade aan de waterzijde
- Dieptelijnen van de bestaande bodem niet meer door het havengebied (zoals in Haven_DO1.dxf)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Onderbouwing/Rekenboek_herontwerp_bijgewerkt.xlsx
+++ b/Onderbouwing/Rekenboek_herontwerp_bijgewerkt.xlsx
@@ -10499,7 +10499,7 @@
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>DO: bekkens + voorhaven, bodemmodel GEBCO 2026 + Copernicus DEM (negatief = boven MLWS, land wordt ontgraven). Celmethode met dieptezones (-18,20/-16,20/-13,70): 61.936.560 m3</t>
+          <t>DO: bekkens + voorhaven, bodemmodel GEBCO 2026 + Copernicus DEM (negatief = boven MLWS, land wordt ontgraven). Celmethode met dieptezones (-18,20/-16,20/-13,70): 61.936.561 m3</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10923,7 @@
       <c r="E24" s="32" t="n"/>
       <c r="F24" s="32" t="inlineStr">
         <is>
-          <t>Aanname. Celmethode: ophoging 354.822 m3, afgraving 7.346.330 m3 (terrein ligt grotendeels hoger dan +5,0 m).</t>
+          <t>Aanname. Celmethode: ophoging 355.044 m3, afgraving 7.346.682 m3 (terrein ligt grotendeels hoger dan +5,0 m).</t>
         </is>
       </c>
       <c r="G24" s="13" t="n"/>

</xml_diff>